<commit_message>
auto: actualizando historial de vacantes
</commit_message>
<xml_diff>
--- a/nuevas_plazas.xlsx
+++ b/nuevas_plazas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O396"/>
+  <dimension ref="A1:O413"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30081,52 +30081,1359 @@
           <t>05/09/2026 a las 09:58</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr">
+      <c r="F396" t="n">
+        <v>28</v>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>Occidente</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>I. E. OLAYA</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>I. E. LLANADAS</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>CORREG. LLANADAS</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t>ón: CRA. 11 10-14</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Cargo Docente tutor (Planta Temporal PTA)</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Primaria</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Frontino</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:14</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>Frontino</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>I. E. R. LA BLANQUITA DEL MURRI</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>I. E. R. LA BLANQUITA DEL MURRI - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>CORREG. LA BLANQUITA MURRI</t>
+        </is>
+      </c>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t>ón: CORREG. LA BLANQUITA MURRI</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Cargo Docente tutor (Planta Temporal PTA)</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Primaria</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Necoclí</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:14</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="G396" t="inlineStr">
-        <is>
-          <t>Occidente</t>
-        </is>
-      </c>
-      <c r="H396" t="inlineStr">
-        <is>
-          <t>Antioquia</t>
-        </is>
-      </c>
-      <c r="I396" t="inlineStr">
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>Necoclí</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
         <is>
           <t>ía de Educación: Antioquia</t>
         </is>
       </c>
-      <c r="J396" t="inlineStr">
-        <is>
-          <t>I. E. OLAYA</t>
-        </is>
-      </c>
-      <c r="K396" t="inlineStr">
-        <is>
-          <t>I. E. LLANADAS</t>
-        </is>
-      </c>
-      <c r="L396" t="inlineStr">
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>I. E. R. PUEBLO NUEVO</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>COLEGIO PUEBLO NUEVO - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
         <is>
           <t>RURAL</t>
         </is>
       </c>
-      <c r="M396" t="inlineStr">
-        <is>
-          <t>CORREG. LLANADAS</t>
-        </is>
-      </c>
-      <c r="N396" t="inlineStr">
-        <is>
-          <t>ón: CRA. 11 10-14</t>
-        </is>
-      </c>
-      <c r="O396" t="inlineStr">
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>CORREG.PUEBLO NUEVO</t>
+        </is>
+      </c>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t>ón: CORREG. PUEBLO NUEVO</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Cargo Docente tutor (Planta Temporal PTA)</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Caucasia</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:14</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>Caucasia</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>I.E. SANTA TERESITA</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>E U SANTA TERESITA - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>URBANA</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t>ón: CLL 19 CRA 6 A 8-6</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Cargo Docente tutor (Planta Temporal PTA)</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Primaria</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Necoclí</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:14</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>Necoclí</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>I.E.R. MELLO VILLAVICENCIO</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>I.E.R MELLOVILLAVICENCIO -SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>CORREG. MELLO VILLAVICENCIO</t>
+        </is>
+      </c>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t>ón: CORREG. MELLO VILLAVICENCIO</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Educación ética y en valores</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Segovia</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:16</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>Segovia</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>I. E. LIBORIO BATALLER</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>C.E.R CUTURU MEDIO</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>Dirección: VDA CUTURU MEDIO</t>
+        </is>
+      </c>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t>ón: VDA CUTURU MEDIO</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Primaria</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Valdivia</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:16</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>Valdivia</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>C. E. R. LA PAULINA</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>C. E. R. LA BARCA CAUTIVA</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>VDA. PTO. RAUDAL</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t>ón: VDA PTO. RAUDAL</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Matemáticas</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Urrao</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:16</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>Urrao</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>I. E. MONSENOR J. IVAN CADAVID GUTIERREZ</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>COLEGIO SIMON BOLIVAR - MONSENOR J. IVAN SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>URBANA</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>BARRIO. INDICIO</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t>ón: CL. 25 Nº 29-41</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Ciencias sociales</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Cáceres</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>Cáceres</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>I. E. R. EL TIGRE</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>C.E.R. SAN PABLO</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t>ón: VEREDA SAN PABLO</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Ciencias naturales y educación ambiental</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>Guadalupe</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>I. E. LUIS LOPEZ DE MESA</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>I. E. R. LA BRAMADORA</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>VDA. GUADALUPE IV</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t>ón: VDA GUADALUPE IV</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Humanidades y lengua castellana</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Frontino</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Frontino</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>I. E. R. LA BLANQUITA DEL MURRI</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>C. E. R. ALTO DE MURRI</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>CORREG DE MURRI</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t>ón: CORREG DE MURRI</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Priorizadas para jóvenes entre 18 y 28 años</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Preescolar</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>San Pedro De Urabá</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>San Pedro de Urabá</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>I.E.R. SAN PABLO APOSTOL</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>I. E. R. SAN PABLO APOSTOL - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>VDA. EL CAIMAN</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t>ón: VDA. EL CAIMÁN</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Educación artística – música</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Arboletes</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Arboletes</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>I. E. R. GUADUAL ARRIBA</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>I. E. R. GUADUAL ARRIBA - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>CORREG. GUADUAL ARRIBA</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t>ón: CORREG. GUADUAL ARRIBA</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Preescolar</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Vigia Del Fuerte</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Vigia del Fuerte</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>I. E. R. ALIANZA PARA EL PROGRESO</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>C. E. R. ISLETA</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>VDA. ISLETA</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t>ón: VDA ISLETA</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Priorizadas para jóvenes entre 18 y 28 años</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Educación artística – música</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>San Pedro De Urabá</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>San Pedro de Urabá</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>I. E. R. SANTA CATALINA</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>COLEGIO SANTA CATALINA - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>CORREG. SANTA CATALINA</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t>ón: CORREG. SANTA CATALINA.</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Preescolar</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Carepa</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>Carepa</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>I. E. COLOMBIA</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>COLEGIO COLOMBIA - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t>URBANA</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>B. GAITAN</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t>ón: CL. 83 CRA67</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Tecnología e informática</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>El Bagre</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:17</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>El Bagre</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>I. E. LA ESMERALDA</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>COLEGIO LA ESMERALDA - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t>URBANA</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>BARRIO LA ESMERALDA</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t>ón: KR 38 69 B 75</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Cargo Docente de aula</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>ón: Vacantes Generales</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Educación física, recreación y deporte</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>El Santuario</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>10/09/2026 a las 09:18</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>Oriente</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>ía de Educación: Antioquia</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>C. E. R. JOSE IGNACIO BOTERO PALACIO</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>C. E. R. JOSE IGNACIO BOTERO PALACIO - SEDE PRINCIPAL</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t>RURAL</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>VDA. VALLE DE MARIA</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t>ón: VDA. VALLE DE MARIA</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>